<commit_message>
Excel in the firm's full 9-sheet format (Gold Star draft layout)
- Template = blank copy of the firm's draft: Facility sanctioned, DP
  calculation, Stock / Debtors / Creditors Holding, Invoice, summation,
  Insurance, GST (GST taxable summary + review stay at the end)
- New sheets filled from the documents: CC outstanding from the bank
  statement, SS and books stock / debtors / creditors, debtor ageing
  (<90 / >90 from SS Annexure IV and the books ageing file), sister
  concerns from the related parties, Tally purchase accounts, GSTR-3B
  sales; holding rows quarterly or monthly as the stock dates fall
- Check page: other facilities, second bank's facility, audited-year
  figures; typed text that is not a number no longer breaks the Excel
- Gold Star vs the firm's draft: 862 / 1072 cells (Facility 100%, DP 99%)

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/template.xlsx
+++ b/docs/template.xlsx
@@ -3,12 +3,18 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr codeName="ThisWorkbook"/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="0" windowWidth="15360" windowHeight="7755" tabRatio="899" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="0" windowWidth="15360" windowHeight="7755" tabRatio="899" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="summation" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Insurance" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="GST" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Facility sanctioned" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DP calculation" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stock Holding" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Debtors Holding" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Creditors Holding" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Invoice" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="summation" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Insurance" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="GST" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="152511" fullCalcOnLoad="1"/>
@@ -851,7 +857,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="294">
+  <cellXfs count="316">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -1537,8 +1543,71 @@
     <xf numFmtId="0" fontId="29" fillId="36" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="1"/>
+    <xf numFmtId="164" fontId="29" fillId="36" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="14" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="16" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="43" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="164" fontId="29" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="43" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="29" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="1"/>
+    <xf numFmtId="166" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
+      <alignment horizontal="right" vertical="top"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
+      <alignment horizontal="right" vertical="top"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="6" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
       <alignment horizontal="right" vertical="top" wrapText="1"/>
     </xf>
@@ -1549,12 +1618,6 @@
     <xf numFmtId="164" fontId="29" fillId="36" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="164" fontId="31" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
@@ -1567,7 +1630,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1577,11 +1639,9 @@
     <xf numFmtId="164" fontId="31" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="1"/>
     <xf numFmtId="164" fontId="31" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="1"/>
   </cellXfs>
   <cellStyles count="81">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2239,6 +2299,1728 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr codeName="Sheet1">
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F16"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="30.5703125" defaultRowHeight="15"/>
+  <cols>
+    <col width="21.5703125" customWidth="1" style="235" min="1" max="1"/>
+    <col width="11" customWidth="1" style="235" min="2" max="2"/>
+    <col width="10.5703125" customWidth="1" style="235" min="3" max="3"/>
+    <col width="10.7109375" customWidth="1" style="235" min="4" max="4"/>
+    <col width="9.7109375" customWidth="1" style="235" min="5" max="5"/>
+    <col width="10.85546875" customWidth="1" style="235" min="6" max="6"/>
+    <col width="27.140625" customWidth="1" style="235" min="7" max="7"/>
+    <col width="15.28515625" customWidth="1" style="235" min="8" max="8"/>
+    <col width="12.42578125" customWidth="1" style="235" min="9" max="9"/>
+    <col width="12.28515625" customWidth="1" style="235" min="10" max="10"/>
+    <col width="16.5703125" customWidth="1" style="235" min="11" max="11"/>
+    <col width="12.7109375" customWidth="1" style="235" min="12" max="12"/>
+    <col width="15.85546875" customWidth="1" style="235" min="13" max="13"/>
+    <col width="30.5703125" customWidth="1" style="235" min="14" max="16"/>
+    <col hidden="1" style="235" min="17" max="17"/>
+    <col width="30.5703125" customWidth="1" style="235" min="18" max="18"/>
+    <col hidden="1" style="235" min="19" max="19"/>
+    <col width="30.5703125" customWidth="1" style="235" min="20" max="16384"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="247" t="n"/>
+    </row>
+    <row r="2" ht="15" customFormat="1" customHeight="1" s="7">
+      <c r="A2" s="248" t="n"/>
+      <c r="B2" s="248" t="n"/>
+      <c r="C2" s="248" t="n"/>
+      <c r="D2" s="275" t="n"/>
+      <c r="E2" s="248" t="n"/>
+      <c r="F2" s="275" t="n"/>
+    </row>
+    <row r="3" ht="15" customFormat="1" customHeight="1" s="7">
+      <c r="A3" s="166" t="n"/>
+      <c r="B3" s="166" t="n"/>
+      <c r="C3" s="248" t="n"/>
+      <c r="D3" s="248" t="n"/>
+      <c r="E3" s="248" t="n"/>
+      <c r="F3" s="248" t="n"/>
+    </row>
+    <row r="4" customFormat="1" s="7">
+      <c r="A4" s="244" t="n"/>
+      <c r="B4" s="276" t="n"/>
+      <c r="C4" s="103" t="n"/>
+      <c r="D4" s="276" t="n"/>
+      <c r="E4" s="73" t="n"/>
+      <c r="F4" s="276" t="n"/>
+    </row>
+    <row r="5" customFormat="1" s="7">
+      <c r="A5" s="244" t="n"/>
+      <c r="B5" s="276" t="n"/>
+      <c r="C5" s="236" t="n"/>
+      <c r="D5" s="276" t="n"/>
+      <c r="E5" s="236" t="n"/>
+      <c r="F5" s="276" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="196" t="n"/>
+      <c r="B6" s="277" t="n"/>
+      <c r="C6" s="277" t="n"/>
+      <c r="D6" s="277" t="n"/>
+      <c r="E6" s="277" t="n"/>
+      <c r="F6" s="277" t="n"/>
+    </row>
+    <row r="7"/>
+    <row r="8"/>
+    <row r="9"/>
+    <row r="10">
+      <c r="A10" s="246" t="n"/>
+      <c r="B10" s="248" t="n"/>
+    </row>
+    <row r="11" ht="15" customHeight="1" s="235">
+      <c r="A11" s="166" t="n"/>
+      <c r="B11" s="166" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="166" t="n"/>
+      <c r="B12" s="244" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="244" t="n"/>
+      <c r="B13" s="244" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="166" t="n"/>
+      <c r="B14" s="244" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="166" t="n"/>
+      <c r="B15" s="244" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="244" t="n"/>
+      <c r="B16" s="244" t="n"/>
+    </row>
+    <row r="21" ht="15" customHeight="1" s="235"/>
+  </sheetData>
+  <mergeCells count="7">
+    <mergeCell ref="C2:D2"/>
+    <mergeCell ref="E2:F2"/>
+    <mergeCell ref="A10:A11"/>
+    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="B2:B3"/>
+    <mergeCell ref="A2:A3"/>
+    <mergeCell ref="B10:B11"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr codeName="Sheet2">
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I92"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="2.85546875" customWidth="1" style="235" min="1" max="1"/>
+    <col width="34.140625" customWidth="1" style="235" min="2" max="2"/>
+    <col width="20.7109375" customWidth="1" style="235" min="3" max="3"/>
+    <col width="20.28515625" customWidth="1" style="235" min="4" max="4"/>
+    <col width="23.140625" customWidth="1" style="235" min="5" max="5"/>
+    <col width="16" customWidth="1" style="235" min="6" max="6"/>
+    <col width="14.28515625" bestFit="1" customWidth="1" style="235" min="7" max="7"/>
+    <col width="14.28515625" customWidth="1" style="235" min="8" max="8"/>
+    <col width="9.140625" customWidth="1" style="235" min="9" max="16384"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="E1" s="2" t="n"/>
+    </row>
+    <row r="2" ht="45" customHeight="1" s="235">
+      <c r="B2" s="248" t="n"/>
+      <c r="C2" s="248" t="n"/>
+      <c r="D2" s="248" t="n"/>
+      <c r="E2" s="248" t="n"/>
+    </row>
+    <row r="3" ht="15" customHeight="1" s="235">
+      <c r="B3" s="111" t="n"/>
+      <c r="C3" s="199" t="n"/>
+      <c r="D3" s="199" t="n"/>
+      <c r="E3" s="199" t="n"/>
+      <c r="G3" s="104" t="n"/>
+    </row>
+    <row r="4" ht="15" customHeight="1" s="235">
+      <c r="B4" s="110" t="n"/>
+      <c r="C4" s="136" t="n"/>
+      <c r="D4" s="136" t="n"/>
+      <c r="E4" s="136" t="n"/>
+      <c r="G4" s="169" t="n"/>
+      <c r="H4" s="278" t="n"/>
+    </row>
+    <row r="5" ht="15" customHeight="1" s="235">
+      <c r="B5" s="111" t="n"/>
+      <c r="C5" s="199" t="n"/>
+      <c r="D5" s="199" t="n"/>
+      <c r="E5" s="199" t="n"/>
+      <c r="F5" s="278" t="n"/>
+      <c r="G5" s="104" t="n"/>
+      <c r="H5" s="278" t="n"/>
+    </row>
+    <row r="6" ht="15" customHeight="1" s="235">
+      <c r="B6" s="110" t="n"/>
+      <c r="C6" s="136" t="n"/>
+      <c r="D6" s="136" t="n"/>
+      <c r="E6" s="136" t="n"/>
+      <c r="F6" s="278" t="n"/>
+      <c r="H6" s="278" t="n"/>
+    </row>
+    <row r="7" ht="15" customHeight="1" s="235">
+      <c r="B7" s="111" t="n"/>
+      <c r="C7" s="199" t="n"/>
+      <c r="D7" s="199" t="n"/>
+      <c r="E7" s="199" t="n"/>
+      <c r="H7" s="278" t="n"/>
+    </row>
+    <row r="8" ht="15" customHeight="1" s="235">
+      <c r="B8" s="111" t="n"/>
+      <c r="C8" s="199" t="n"/>
+      <c r="D8" s="199" t="n"/>
+      <c r="E8" s="199" t="n"/>
+      <c r="G8" s="194" t="n"/>
+      <c r="H8" s="278" t="n"/>
+    </row>
+    <row r="9" ht="15" customHeight="1" s="235">
+      <c r="B9" s="111" t="n"/>
+      <c r="C9" s="199" t="n"/>
+      <c r="D9" s="203" t="n"/>
+      <c r="E9" s="199" t="n"/>
+      <c r="H9" s="278" t="n"/>
+    </row>
+    <row r="10" ht="15" customHeight="1" s="235">
+      <c r="B10" s="244" t="n"/>
+      <c r="C10" s="73" t="n"/>
+      <c r="D10" s="73" t="n"/>
+      <c r="E10" s="73" t="n"/>
+      <c r="H10" s="278" t="n"/>
+    </row>
+    <row r="11" ht="15" customHeight="1" s="235">
+      <c r="B11" s="204" t="n"/>
+      <c r="C11" s="205" t="n"/>
+      <c r="D11" s="205" t="n"/>
+      <c r="E11" s="205" t="n"/>
+      <c r="H11" s="278" t="n"/>
+    </row>
+    <row r="12" ht="15" customHeight="1" s="235">
+      <c r="B12" s="110" t="n"/>
+      <c r="C12" s="114" t="n"/>
+      <c r="D12" s="114" t="n"/>
+      <c r="E12" s="114" t="n"/>
+      <c r="H12" s="169" t="n"/>
+    </row>
+    <row r="13" ht="15" customHeight="1" s="235">
+      <c r="B13" s="111" t="n"/>
+      <c r="C13" s="203" t="n"/>
+      <c r="D13" s="203" t="n"/>
+      <c r="E13" s="203" t="n"/>
+      <c r="H13" s="169" t="n"/>
+    </row>
+    <row r="14" ht="30" customHeight="1" s="235">
+      <c r="B14" s="111" t="n"/>
+      <c r="C14" s="203" t="n"/>
+      <c r="D14" s="203" t="n"/>
+      <c r="E14" s="203" t="n"/>
+      <c r="H14" s="169" t="n"/>
+    </row>
+    <row r="15" ht="15" customHeight="1" s="235">
+      <c r="B15" s="111" t="n"/>
+      <c r="C15" s="199" t="n"/>
+      <c r="D15" s="199" t="n"/>
+      <c r="E15" s="199" t="n"/>
+      <c r="H15" s="169" t="n"/>
+      <c r="I15" s="195" t="n"/>
+    </row>
+    <row r="16" ht="15" customHeight="1" s="235">
+      <c r="B16" s="111" t="n"/>
+      <c r="C16" s="199" t="n"/>
+      <c r="D16" s="199" t="n"/>
+      <c r="E16" s="199" t="n"/>
+      <c r="H16" s="169" t="n"/>
+    </row>
+    <row r="17" ht="15" customHeight="1" s="235">
+      <c r="B17" s="111" t="n"/>
+      <c r="C17" s="199" t="n"/>
+      <c r="D17" s="199" t="n"/>
+      <c r="E17" s="199" t="n"/>
+      <c r="H17" s="169" t="n"/>
+    </row>
+    <row r="18" ht="15" customHeight="1" s="235">
+      <c r="B18" s="111" t="n"/>
+      <c r="C18" s="199" t="n"/>
+      <c r="D18" s="199" t="n"/>
+      <c r="E18" s="199" t="n"/>
+      <c r="H18" s="169" t="n"/>
+    </row>
+    <row r="19" ht="15" customHeight="1" s="235">
+      <c r="B19" s="111" t="n"/>
+      <c r="C19" s="199" t="n"/>
+      <c r="D19" s="199" t="n"/>
+      <c r="E19" s="199" t="n"/>
+      <c r="H19" s="169" t="n"/>
+    </row>
+    <row r="20" ht="15" customHeight="1" s="235">
+      <c r="B20" s="111" t="n"/>
+      <c r="C20" s="199" t="n"/>
+      <c r="D20" s="199" t="n"/>
+      <c r="E20" s="199" t="n"/>
+      <c r="H20" s="169" t="n"/>
+    </row>
+    <row r="21" ht="15" customHeight="1" s="235">
+      <c r="B21" s="111" t="n"/>
+      <c r="C21" s="199" t="n"/>
+      <c r="D21" s="199" t="n"/>
+      <c r="E21" s="199" t="n"/>
+      <c r="H21" s="169" t="n"/>
+    </row>
+    <row r="22" ht="15" customHeight="1" s="235">
+      <c r="B22" s="111" t="n"/>
+      <c r="C22" s="199" t="n"/>
+      <c r="D22" s="199" t="n"/>
+      <c r="E22" s="199" t="n"/>
+      <c r="H22" s="169" t="n"/>
+    </row>
+    <row r="23" ht="15" customHeight="1" s="235">
+      <c r="B23" s="111" t="n"/>
+      <c r="C23" s="115" t="n"/>
+      <c r="D23" s="115" t="n"/>
+      <c r="E23" s="115" t="n"/>
+      <c r="H23" s="10" t="n"/>
+    </row>
+    <row r="24" ht="15" customHeight="1" s="235">
+      <c r="B24" s="204" t="n"/>
+      <c r="C24" s="217" t="n"/>
+      <c r="D24" s="217" t="n"/>
+      <c r="E24" s="217" t="n"/>
+      <c r="H24" s="10" t="n"/>
+    </row>
+    <row r="25" ht="15" customHeight="1" s="235">
+      <c r="B25" s="7" t="n"/>
+      <c r="C25" s="194" t="n"/>
+      <c r="D25" s="194" t="n"/>
+      <c r="E25" s="194" t="n"/>
+      <c r="H25" s="10" t="n"/>
+    </row>
+    <row r="26" ht="15" customHeight="1" s="235">
+      <c r="B26" s="248" t="n"/>
+      <c r="C26" s="248" t="n"/>
+      <c r="D26" s="248" t="n"/>
+      <c r="E26" s="248" t="n"/>
+      <c r="H26" s="10" t="n"/>
+    </row>
+    <row r="27" ht="15" customHeight="1" s="235">
+      <c r="B27" s="163" t="n"/>
+      <c r="C27" s="136" t="n"/>
+      <c r="D27" s="136" t="n"/>
+      <c r="E27" s="73" t="n"/>
+    </row>
+    <row r="28" ht="15" customHeight="1" s="235">
+      <c r="B28" s="163" t="n"/>
+      <c r="C28" s="136" t="n"/>
+      <c r="D28" s="136" t="n"/>
+      <c r="E28" s="73" t="n"/>
+    </row>
+    <row r="29" ht="15" customHeight="1" s="235">
+      <c r="B29" s="163" t="n"/>
+      <c r="C29" s="136" t="n"/>
+      <c r="D29" s="136" t="n"/>
+      <c r="E29" s="73" t="n"/>
+    </row>
+    <row r="30" ht="15" customHeight="1" s="235">
+      <c r="B30" s="106" t="n"/>
+      <c r="C30" s="279" t="n"/>
+      <c r="D30" s="279" t="n"/>
+    </row>
+    <row r="31" ht="15" customHeight="1" s="235">
+      <c r="B31" s="248" t="n"/>
+      <c r="C31" s="248" t="n"/>
+      <c r="D31" s="138" t="n"/>
+    </row>
+    <row r="32" ht="15" customHeight="1" s="235">
+      <c r="B32" s="163" t="n"/>
+      <c r="C32" s="280" t="n"/>
+      <c r="D32" s="154" t="n"/>
+      <c r="E32" s="154" t="n"/>
+    </row>
+    <row r="33" ht="15" customHeight="1" s="235">
+      <c r="B33" s="163" t="n"/>
+      <c r="C33" s="280" t="n"/>
+      <c r="D33" s="154" t="n"/>
+      <c r="E33" s="154" t="n"/>
+    </row>
+    <row r="34" ht="15" customHeight="1" s="235">
+      <c r="B34" s="163" t="n"/>
+      <c r="C34" s="280" t="n"/>
+      <c r="D34" s="154" t="n"/>
+      <c r="E34" s="154" t="n"/>
+    </row>
+    <row r="35" ht="15" customHeight="1" s="235">
+      <c r="B35" s="106" t="n"/>
+      <c r="C35" s="279" t="n"/>
+      <c r="D35" s="279" t="n"/>
+    </row>
+    <row r="36"/>
+    <row r="37"/>
+    <row r="38" ht="30" customHeight="1" s="235">
+      <c r="B38" s="251" t="n"/>
+      <c r="C38" s="251" t="n"/>
+      <c r="D38" s="251" t="n"/>
+      <c r="E38" s="251" t="n"/>
+    </row>
+    <row r="39">
+      <c r="B39" s="94" t="n"/>
+      <c r="C39" s="107" t="n"/>
+      <c r="D39" s="107" t="n"/>
+      <c r="E39" s="151" t="n"/>
+      <c r="F39" s="194" t="n"/>
+    </row>
+    <row r="40">
+      <c r="B40" s="97" t="n"/>
+      <c r="C40" s="108" t="n"/>
+      <c r="D40" s="108" t="n"/>
+      <c r="E40" s="108" t="n"/>
+    </row>
+    <row r="41" ht="15.75" customHeight="1" s="235">
+      <c r="B41" s="251" t="n"/>
+      <c r="C41" s="251" t="n"/>
+      <c r="D41" s="275" t="n"/>
+      <c r="E41" s="251" t="n"/>
+      <c r="F41" s="275" t="n"/>
+    </row>
+    <row r="42">
+      <c r="B42" s="166" t="n"/>
+      <c r="C42" s="251" t="n"/>
+      <c r="D42" s="251" t="n"/>
+      <c r="E42" s="251" t="n"/>
+      <c r="F42" s="251" t="n"/>
+    </row>
+    <row r="43">
+      <c r="B43" s="145" t="n"/>
+      <c r="C43" s="281" t="n"/>
+      <c r="D43" s="281" t="n"/>
+      <c r="E43" s="281" t="n"/>
+      <c r="F43" s="281" t="n"/>
+      <c r="G43" s="195" t="n"/>
+      <c r="H43" s="195" t="n"/>
+    </row>
+    <row r="44">
+      <c r="B44" s="266" t="n"/>
+      <c r="C44" s="281" t="n"/>
+      <c r="D44" s="281" t="n"/>
+      <c r="E44" s="281" t="n"/>
+      <c r="F44" s="281" t="n"/>
+    </row>
+    <row r="45">
+      <c r="B45" s="266" t="n"/>
+      <c r="C45" s="281" t="n"/>
+      <c r="D45" s="281" t="n"/>
+      <c r="E45" s="281" t="n"/>
+      <c r="F45" s="281" t="n"/>
+      <c r="G45" s="195" t="n"/>
+      <c r="H45" s="195" t="n"/>
+    </row>
+    <row r="46">
+      <c r="B46" s="230" t="n"/>
+      <c r="C46" s="108" t="n"/>
+      <c r="D46" s="108" t="n"/>
+      <c r="E46" s="108" t="n"/>
+      <c r="F46" s="108" t="n"/>
+    </row>
+    <row r="47"/>
+    <row r="48">
+      <c r="B48" s="146" t="n"/>
+      <c r="C48" s="147" t="n"/>
+      <c r="D48" s="147" t="n"/>
+      <c r="E48" s="147" t="n"/>
+    </row>
+    <row r="49">
+      <c r="B49" s="222" t="n"/>
+      <c r="C49" s="73" t="n"/>
+      <c r="D49" s="73" t="n"/>
+      <c r="E49" s="191" t="n"/>
+      <c r="F49" s="194" t="n"/>
+    </row>
+    <row r="50">
+      <c r="B50" s="263" t="n"/>
+      <c r="C50" s="73" t="n"/>
+      <c r="D50" s="68" t="n"/>
+      <c r="E50" s="191" t="n"/>
+      <c r="F50" s="194" t="n"/>
+    </row>
+    <row r="51">
+      <c r="B51" s="84" t="n"/>
+      <c r="C51" s="73" t="n"/>
+      <c r="D51" s="73" t="n"/>
+      <c r="E51" s="191" t="n"/>
+      <c r="F51" s="194" t="n"/>
+    </row>
+    <row r="52">
+      <c r="B52" s="150" t="n"/>
+      <c r="C52" s="194" t="n"/>
+      <c r="D52" s="194" t="n"/>
+      <c r="E52" s="195" t="n"/>
+      <c r="F52" s="194" t="n"/>
+    </row>
+    <row r="53"/>
+    <row r="54">
+      <c r="B54" s="146" t="n"/>
+      <c r="C54" s="147" t="n"/>
+      <c r="D54" s="147" t="n"/>
+      <c r="E54" s="147" t="n"/>
+    </row>
+    <row r="55">
+      <c r="B55" s="222" t="n"/>
+      <c r="C55" s="68" t="n"/>
+      <c r="D55" s="68" t="n"/>
+      <c r="E55" s="191" t="n"/>
+      <c r="F55" s="194" t="n"/>
+    </row>
+    <row r="56">
+      <c r="B56" s="263" t="n"/>
+      <c r="C56" s="68" t="n"/>
+      <c r="D56" s="68" t="n"/>
+      <c r="E56" s="191" t="n"/>
+      <c r="F56" s="194" t="n"/>
+    </row>
+    <row r="57">
+      <c r="B57" s="84" t="n"/>
+      <c r="C57" s="68" t="n"/>
+      <c r="D57" s="282" t="n"/>
+      <c r="E57" s="191" t="n"/>
+      <c r="F57" s="194" t="n"/>
+    </row>
+    <row r="58">
+      <c r="C58" s="194" t="n"/>
+      <c r="D58" s="194" t="n"/>
+      <c r="E58" s="195" t="n"/>
+      <c r="F58" s="194" t="n"/>
+    </row>
+    <row r="59"/>
+    <row r="60"/>
+    <row r="61"/>
+    <row r="62"/>
+    <row r="63"/>
+    <row r="64">
+      <c r="B64" s="138" t="n"/>
+      <c r="C64" s="138" t="n"/>
+      <c r="D64" s="138" t="n"/>
+      <c r="E64" s="138" t="n"/>
+    </row>
+    <row r="65">
+      <c r="B65" s="173" t="n"/>
+      <c r="C65" s="174" t="n"/>
+      <c r="D65" s="174" t="n"/>
+      <c r="E65" s="174" t="n"/>
+    </row>
+    <row r="66">
+      <c r="B66" s="175" t="n"/>
+      <c r="C66" s="176" t="n"/>
+      <c r="D66" s="176" t="n"/>
+      <c r="E66" s="176" t="n"/>
+    </row>
+    <row r="67">
+      <c r="B67" s="173" t="n"/>
+      <c r="C67" s="174" t="n"/>
+      <c r="D67" s="174" t="n"/>
+      <c r="E67" s="174" t="n"/>
+    </row>
+    <row r="68"/>
+    <row r="69"/>
+    <row r="70"/>
+    <row r="71"/>
+    <row r="72"/>
+    <row r="73"/>
+    <row r="74"/>
+    <row r="75"/>
+    <row r="76"/>
+    <row r="77"/>
+    <row r="78"/>
+    <row r="79"/>
+    <row r="80"/>
+    <row r="81"/>
+    <row r="82"/>
+    <row r="83"/>
+    <row r="84"/>
+    <row r="85"/>
+    <row r="86"/>
+    <row r="87"/>
+    <row r="88"/>
+    <row r="89"/>
+    <row r="90"/>
+    <row r="91"/>
+    <row r="92"/>
+  </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="B41:B42"/>
+    <mergeCell ref="E41:F41"/>
+    <mergeCell ref="C41:D41"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr codeName="Sheet3">
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:W64"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="23.7109375" customWidth="1" style="235" min="1" max="1"/>
+    <col width="16.5703125" customWidth="1" style="235" min="2" max="3"/>
+    <col width="16.85546875" customWidth="1" style="235" min="4" max="4"/>
+    <col width="19.7109375" bestFit="1" customWidth="1" style="235" min="5" max="5"/>
+    <col width="16.85546875" bestFit="1" customWidth="1" style="235" min="6" max="6"/>
+    <col width="10.28515625" customWidth="1" style="235" min="7" max="7"/>
+    <col width="15.85546875" bestFit="1" customWidth="1" style="235" min="8" max="8"/>
+    <col width="14.42578125" bestFit="1" customWidth="1" style="235" min="9" max="9"/>
+    <col width="12.7109375" bestFit="1" customWidth="1" style="235" min="10" max="10"/>
+    <col width="9.140625" customWidth="1" style="235" min="11" max="11"/>
+    <col width="14.28515625" bestFit="1" customWidth="1" style="235" min="12" max="12"/>
+    <col width="15.85546875" bestFit="1" customWidth="1" style="235" min="13" max="13"/>
+    <col width="14.7109375" bestFit="1" customWidth="1" style="235" min="14" max="14"/>
+    <col width="10.42578125" bestFit="1" customWidth="1" style="235" min="15" max="15"/>
+    <col width="12" bestFit="1" customWidth="1" style="235" min="16" max="16"/>
+    <col width="14.42578125" bestFit="1" customWidth="1" style="235" min="17" max="17"/>
+    <col width="14.42578125" customWidth="1" style="235" min="18" max="18"/>
+    <col width="14.42578125" bestFit="1" customWidth="1" style="235" min="19" max="19"/>
+    <col width="14.42578125" customWidth="1" style="235" min="20" max="20"/>
+    <col width="9.140625" customWidth="1" style="235" min="21" max="21"/>
+    <col width="9.140625" customWidth="1" style="235" min="22" max="16384"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="258" t="n"/>
+      <c r="B1" s="283" t="n"/>
+      <c r="C1" s="283" t="n"/>
+      <c r="D1" s="283" t="n"/>
+      <c r="E1" s="283" t="n"/>
+      <c r="F1" s="283" t="n"/>
+      <c r="G1" s="283" t="n"/>
+      <c r="H1" s="283" t="n"/>
+      <c r="I1" s="283" t="n"/>
+      <c r="J1" s="283" t="n"/>
+      <c r="U1" s="257" t="n"/>
+    </row>
+    <row r="2">
+      <c r="A2" s="248" t="n"/>
+      <c r="B2" s="251" t="n"/>
+      <c r="C2" s="248" t="n"/>
+      <c r="D2" s="248" t="n"/>
+      <c r="E2" s="248" t="n"/>
+      <c r="F2" s="248" t="n"/>
+      <c r="H2" s="244" t="n"/>
+      <c r="I2" s="87" t="n"/>
+      <c r="J2" s="87" t="n"/>
+      <c r="K2" s="87" t="n"/>
+      <c r="L2" s="170" t="n"/>
+      <c r="M2" s="170" t="n"/>
+      <c r="N2" s="167" t="n"/>
+      <c r="O2" s="167" t="n"/>
+      <c r="P2" s="167" t="n"/>
+      <c r="Q2" s="167" t="n"/>
+      <c r="R2" s="167" t="n"/>
+      <c r="S2" s="167" t="n"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="54" t="n"/>
+      <c r="B3" s="200" t="n"/>
+      <c r="C3" s="73" t="n"/>
+      <c r="D3" s="200" t="n"/>
+      <c r="E3" s="200" t="n"/>
+      <c r="F3" s="21" t="n"/>
+      <c r="H3" s="54" t="n"/>
+      <c r="I3" s="200" t="n"/>
+      <c r="J3" s="200" t="n"/>
+      <c r="K3" s="73" t="n"/>
+      <c r="L3" s="194" t="n"/>
+      <c r="M3" s="169" t="n"/>
+      <c r="N3" s="169" t="n"/>
+      <c r="O3" s="169" t="n"/>
+      <c r="P3" s="194" t="n"/>
+      <c r="Q3" s="169" t="n"/>
+      <c r="R3" s="169" t="n"/>
+      <c r="S3" s="169" t="n"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="54" t="n"/>
+      <c r="B4" s="200" t="n"/>
+      <c r="C4" s="73" t="n"/>
+      <c r="D4" s="200" t="n"/>
+      <c r="E4" s="200" t="n"/>
+      <c r="F4" s="21" t="n"/>
+      <c r="H4" s="54" t="n"/>
+      <c r="I4" s="200" t="n"/>
+      <c r="J4" s="200" t="n"/>
+      <c r="K4" s="73" t="n"/>
+      <c r="L4" s="194" t="n"/>
+      <c r="M4" s="169" t="n"/>
+      <c r="N4" s="169" t="n"/>
+      <c r="O4" s="169" t="n"/>
+      <c r="P4" s="194" t="n"/>
+      <c r="Q4" s="169" t="n"/>
+      <c r="R4" s="169" t="n"/>
+      <c r="S4" s="169" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="54" t="n"/>
+      <c r="B5" s="200" t="n"/>
+      <c r="C5" s="73" t="n"/>
+      <c r="D5" s="200" t="n"/>
+      <c r="E5" s="200" t="n"/>
+      <c r="F5" s="21" t="n"/>
+      <c r="H5" s="54" t="n"/>
+      <c r="I5" s="68" t="n"/>
+      <c r="J5" s="200" t="n"/>
+      <c r="K5" s="73" t="n"/>
+      <c r="L5" s="194" t="n"/>
+      <c r="M5" s="169" t="n"/>
+      <c r="N5" s="169" t="n"/>
+      <c r="O5" s="169" t="n"/>
+      <c r="P5" s="194" t="n"/>
+      <c r="Q5" s="169" t="n"/>
+      <c r="R5" s="169" t="n"/>
+      <c r="S5" s="169" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="248" t="n"/>
+      <c r="B6" s="284" t="n"/>
+      <c r="C6" s="284" t="n"/>
+      <c r="D6" s="284" t="n"/>
+      <c r="E6" s="275" t="n"/>
+      <c r="F6" s="86" t="n"/>
+      <c r="J6" s="194" t="n"/>
+      <c r="N6" s="169" t="n"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="6" t="n"/>
+      <c r="B7" s="6" t="n"/>
+      <c r="C7" s="5" t="n"/>
+      <c r="D7" s="6" t="n"/>
+      <c r="E7" s="6" t="n"/>
+      <c r="M7" s="194" t="n"/>
+      <c r="N7" s="194" t="n"/>
+      <c r="O7" s="194" t="n"/>
+      <c r="Q7" s="169" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="6" t="n"/>
+      <c r="B8" s="6" t="n"/>
+      <c r="C8" s="6" t="n"/>
+      <c r="D8" s="6" t="n"/>
+      <c r="E8" s="6" t="n"/>
+      <c r="H8" s="169" t="n"/>
+      <c r="J8" s="169" t="n"/>
+      <c r="M8" s="194" t="n"/>
+      <c r="N8" s="194" t="n"/>
+      <c r="O8" s="194" t="n"/>
+    </row>
+    <row r="9" ht="15" customHeight="1" s="235">
+      <c r="A9" s="251" t="n"/>
+      <c r="B9" s="251" t="n"/>
+      <c r="C9" s="251" t="n"/>
+      <c r="D9" s="251" t="n"/>
+      <c r="G9" s="169" t="n"/>
+      <c r="M9" s="194" t="n"/>
+      <c r="N9" s="194" t="n"/>
+      <c r="O9" s="194" t="n"/>
+    </row>
+    <row r="10" ht="15" customHeight="1" s="235">
+      <c r="A10" s="55" t="n"/>
+      <c r="B10" s="280" t="n"/>
+      <c r="C10" s="280" t="n"/>
+      <c r="D10" s="117" t="n"/>
+      <c r="E10" s="285" t="n"/>
+      <c r="G10" s="169" t="n"/>
+      <c r="M10" s="194" t="n"/>
+      <c r="N10" s="194" t="n"/>
+      <c r="O10" s="194" t="n"/>
+    </row>
+    <row r="11" ht="15" customHeight="1" s="235">
+      <c r="A11" s="88" t="n"/>
+      <c r="B11" s="169" t="n"/>
+      <c r="C11" s="169" t="n"/>
+      <c r="D11" s="90" t="n"/>
+      <c r="E11" s="6" t="n"/>
+      <c r="G11" s="169" t="n"/>
+      <c r="H11" s="194" t="n"/>
+      <c r="J11" s="169" t="n"/>
+      <c r="M11" s="194" t="n"/>
+      <c r="N11" s="194" t="n"/>
+      <c r="O11" s="194" t="n"/>
+    </row>
+    <row r="12" ht="15" customHeight="1" s="235">
+      <c r="A12" s="248" t="n"/>
+      <c r="B12" s="248" t="n"/>
+      <c r="C12" s="248" t="n"/>
+      <c r="D12" s="248" t="n"/>
+      <c r="E12" s="6" t="n"/>
+      <c r="G12" s="169" t="n"/>
+      <c r="H12" s="194" t="n"/>
+      <c r="J12" s="169" t="n"/>
+      <c r="M12" s="194" t="n"/>
+      <c r="N12" s="194" t="n"/>
+      <c r="O12" s="194" t="n"/>
+    </row>
+    <row r="13" ht="15" customHeight="1" s="235">
+      <c r="A13" s="152" t="n"/>
+      <c r="B13" s="286" t="n"/>
+      <c r="C13" s="286" t="n"/>
+      <c r="D13" s="287" t="n"/>
+      <c r="E13" s="6" t="n"/>
+      <c r="G13" s="169" t="n"/>
+      <c r="H13" s="194" t="n"/>
+      <c r="J13" s="169" t="n"/>
+      <c r="M13" s="194" t="n"/>
+      <c r="N13" s="194" t="n"/>
+      <c r="O13" s="194" t="n"/>
+    </row>
+    <row r="14" ht="15" customHeight="1" s="235">
+      <c r="A14" s="152" t="n"/>
+      <c r="B14" s="286" t="n"/>
+      <c r="C14" s="286" t="n"/>
+      <c r="D14" s="287" t="n"/>
+      <c r="E14" s="6" t="n"/>
+      <c r="G14" s="169" t="n"/>
+      <c r="H14" s="194" t="n"/>
+      <c r="J14" s="169" t="n"/>
+      <c r="M14" s="194" t="n"/>
+      <c r="N14" s="194" t="n"/>
+      <c r="O14" s="194" t="n"/>
+    </row>
+    <row r="15" ht="15" customHeight="1" s="235">
+      <c r="A15" s="152" t="n"/>
+      <c r="B15" s="286" t="n"/>
+      <c r="C15" s="286" t="n"/>
+      <c r="D15" s="287" t="n"/>
+      <c r="E15" s="6" t="n"/>
+      <c r="G15" s="169" t="n"/>
+      <c r="H15" s="194" t="n"/>
+      <c r="J15" s="169" t="n"/>
+      <c r="M15" s="194" t="n"/>
+      <c r="N15" s="194" t="n"/>
+      <c r="O15" s="194" t="n"/>
+    </row>
+    <row r="16" ht="15" customHeight="1" s="235">
+      <c r="A16" s="152" t="n"/>
+      <c r="B16" s="286" t="n"/>
+      <c r="C16" s="286" t="n"/>
+      <c r="D16" s="287" t="n"/>
+      <c r="E16" s="6" t="n"/>
+      <c r="G16" s="169" t="n"/>
+      <c r="H16" s="194" t="n"/>
+      <c r="J16" s="169" t="n"/>
+      <c r="M16" s="194" t="n"/>
+      <c r="N16" s="194" t="n"/>
+      <c r="O16" s="194" t="n"/>
+    </row>
+    <row r="17" ht="15" customHeight="1" s="235">
+      <c r="A17" s="152" t="n"/>
+      <c r="B17" s="286" t="n"/>
+      <c r="C17" s="286" t="n"/>
+      <c r="D17" s="287" t="n"/>
+      <c r="E17" s="6" t="n"/>
+      <c r="G17" s="169" t="n"/>
+      <c r="H17" s="194" t="n"/>
+      <c r="J17" s="169" t="n"/>
+    </row>
+    <row r="18" ht="15" customHeight="1" s="235">
+      <c r="A18" s="152" t="n"/>
+      <c r="B18" s="286" t="n"/>
+      <c r="C18" s="286" t="n"/>
+      <c r="D18" s="287" t="n"/>
+      <c r="E18" s="6" t="n"/>
+      <c r="G18" s="169" t="n"/>
+      <c r="H18" s="194" t="n"/>
+      <c r="J18" s="169" t="n"/>
+    </row>
+    <row r="19" ht="15" customHeight="1" s="235">
+      <c r="A19" s="152" t="n"/>
+      <c r="B19" s="286" t="n"/>
+      <c r="C19" s="286" t="n"/>
+      <c r="D19" s="287" t="n"/>
+      <c r="E19" s="6" t="n"/>
+      <c r="G19" s="169" t="n"/>
+      <c r="H19" s="194" t="n"/>
+      <c r="J19" s="169" t="n"/>
+    </row>
+    <row r="20" ht="15" customHeight="1" s="235">
+      <c r="A20" s="88" t="n"/>
+      <c r="B20" s="169" t="n"/>
+      <c r="C20" s="169" t="n"/>
+      <c r="D20" s="90" t="n"/>
+      <c r="E20" s="6" t="n"/>
+      <c r="G20" s="169" t="n"/>
+      <c r="H20" s="194" t="n"/>
+      <c r="J20" s="169" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="248" t="n"/>
+      <c r="B21" s="248" t="n"/>
+      <c r="C21" s="248" t="n"/>
+      <c r="D21" s="248" t="n"/>
+      <c r="H21" s="169" t="n"/>
+      <c r="I21" s="169" t="n"/>
+      <c r="J21" s="169" t="n"/>
+    </row>
+    <row r="22" ht="12.95" customHeight="1" s="235">
+      <c r="A22" s="241" t="n"/>
+      <c r="B22" s="286" t="n"/>
+      <c r="C22" s="286" t="n"/>
+      <c r="D22" s="287" t="n"/>
+      <c r="H22" s="169" t="n"/>
+      <c r="I22" s="169" t="n"/>
+      <c r="J22" s="194" t="n"/>
+    </row>
+    <row r="23" ht="12.95" customHeight="1" s="235">
+      <c r="A23" s="152" t="n"/>
+      <c r="B23" s="286" t="n"/>
+      <c r="C23" s="286" t="n"/>
+      <c r="D23" s="287" t="n"/>
+      <c r="H23" s="169" t="n"/>
+      <c r="I23" s="169" t="n"/>
+      <c r="J23" s="194" t="n"/>
+    </row>
+    <row r="24" ht="12.95" customHeight="1" s="235">
+      <c r="A24" s="152" t="n"/>
+      <c r="B24" s="286" t="n"/>
+      <c r="C24" s="286" t="n"/>
+      <c r="D24" s="287" t="n"/>
+      <c r="H24" s="169" t="n"/>
+      <c r="I24" s="169" t="n"/>
+      <c r="J24" s="194" t="n"/>
+    </row>
+    <row r="25" ht="12.95" customHeight="1" s="235">
+      <c r="A25" s="152" t="n"/>
+      <c r="B25" s="286" t="n"/>
+      <c r="C25" s="286" t="n"/>
+      <c r="D25" s="287" t="n"/>
+      <c r="H25" s="169" t="n"/>
+      <c r="I25" s="169" t="n"/>
+      <c r="J25" s="194" t="n"/>
+    </row>
+    <row r="26" ht="12.95" customHeight="1" s="235">
+      <c r="A26" s="152" t="n"/>
+      <c r="B26" s="286" t="n"/>
+      <c r="C26" s="286" t="n"/>
+      <c r="D26" s="287" t="n"/>
+      <c r="H26" s="169" t="n"/>
+      <c r="I26" s="169" t="n"/>
+      <c r="J26" s="194" t="n"/>
+    </row>
+    <row r="27" ht="12.95" customHeight="1" s="235">
+      <c r="A27" s="152" t="n"/>
+      <c r="B27" s="286" t="n"/>
+      <c r="C27" s="286" t="n"/>
+      <c r="D27" s="287" t="n"/>
+      <c r="H27" s="169" t="n"/>
+      <c r="I27" s="169" t="n"/>
+      <c r="J27" s="194" t="n"/>
+    </row>
+    <row r="28" ht="30" customHeight="1" s="235">
+      <c r="A28" s="266" t="n"/>
+      <c r="B28" s="284" t="n"/>
+      <c r="C28" s="275" t="n"/>
+      <c r="D28" s="288" t="n"/>
+      <c r="H28" s="169" t="n"/>
+      <c r="I28" s="169" t="n"/>
+      <c r="J28" s="194" t="n"/>
+    </row>
+    <row r="29" ht="30" customHeight="1" s="235">
+      <c r="A29" s="266" t="n"/>
+      <c r="B29" s="284" t="n"/>
+      <c r="C29" s="275" t="n"/>
+      <c r="D29" s="288" t="n"/>
+      <c r="H29" s="169" t="n"/>
+      <c r="I29" s="169" t="n"/>
+      <c r="J29" s="194" t="n"/>
+    </row>
+    <row r="30" ht="15" customHeight="1" s="235">
+      <c r="A30" s="266" t="n"/>
+      <c r="B30" s="284" t="n"/>
+      <c r="C30" s="275" t="n"/>
+      <c r="D30" s="288" t="n"/>
+      <c r="H30" s="169" t="n"/>
+      <c r="I30" s="169" t="n"/>
+      <c r="J30" s="194" t="n"/>
+    </row>
+    <row r="31" ht="15" customHeight="1" s="235">
+      <c r="A31" s="266" t="n"/>
+      <c r="B31" s="284" t="n"/>
+      <c r="C31" s="275" t="n"/>
+      <c r="D31" s="151" t="n"/>
+      <c r="H31" s="169" t="n"/>
+      <c r="I31" s="169" t="n"/>
+      <c r="J31" s="194" t="n"/>
+    </row>
+    <row r="32" ht="15" customHeight="1" s="235">
+      <c r="A32" s="230" t="n"/>
+      <c r="B32" s="230" t="n"/>
+      <c r="C32" s="230" t="n"/>
+      <c r="D32" s="230" t="n"/>
+      <c r="H32" s="169" t="n"/>
+      <c r="I32" s="169" t="n"/>
+      <c r="J32" s="194" t="n"/>
+    </row>
+    <row r="33" ht="12.95" customHeight="1" s="235">
+      <c r="A33" s="85" t="n"/>
+      <c r="B33" s="169" t="n"/>
+      <c r="C33" s="169" t="n"/>
+      <c r="D33" s="169" t="n"/>
+      <c r="H33" s="169" t="n"/>
+      <c r="I33" s="169" t="n"/>
+      <c r="J33" s="194" t="n"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="289" t="n"/>
+      <c r="B34" s="6" t="n"/>
+      <c r="C34" s="6" t="n"/>
+      <c r="D34" s="290" t="n"/>
+      <c r="E34" s="290" t="n"/>
+    </row>
+    <row r="35" ht="60" customHeight="1" s="235">
+      <c r="A35" s="248" t="n"/>
+      <c r="B35" s="248" t="n"/>
+      <c r="C35" s="248" t="n"/>
+      <c r="D35" s="248" t="n"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="253" t="n"/>
+      <c r="B36" s="291" t="n"/>
+      <c r="C36" s="291" t="n"/>
+      <c r="D36" s="158" t="n"/>
+      <c r="E36" s="278" t="n"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="16" t="n"/>
+      <c r="B37" s="6" t="n"/>
+      <c r="C37" s="6" t="n"/>
+      <c r="D37" s="292" t="n"/>
+      <c r="E37" s="293" t="n"/>
+    </row>
+    <row r="38"/>
+    <row r="39">
+      <c r="A39" s="252" t="n"/>
+      <c r="B39" s="284" t="n"/>
+      <c r="C39" s="275" t="n"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="248" t="n"/>
+      <c r="B40" s="275" t="n"/>
+      <c r="C40" s="248" t="n"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="253" t="n"/>
+      <c r="B41" s="275" t="n"/>
+      <c r="C41" s="294" t="n"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="252" t="n"/>
+      <c r="B42" s="284" t="n"/>
+      <c r="C42" s="275" t="n"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="248" t="n"/>
+      <c r="B43" s="275" t="n"/>
+      <c r="C43" s="248" t="n"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="253" t="n"/>
+      <c r="B44" s="275" t="n"/>
+      <c r="C44" s="294" t="n"/>
+    </row>
+    <row r="45"/>
+    <row r="46"/>
+    <row r="47">
+      <c r="A47" s="92" t="n"/>
+      <c r="B47" s="91" t="n"/>
+    </row>
+    <row r="48" ht="30" customHeight="1" s="235">
+      <c r="A48" s="266" t="n"/>
+      <c r="B48" s="288" t="n"/>
+    </row>
+    <row r="49" ht="45" customHeight="1" s="235">
+      <c r="A49" s="266" t="n"/>
+      <c r="B49" s="288" t="n"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="266" t="n"/>
+      <c r="B50" s="288" t="n"/>
+      <c r="C50" s="194" t="n"/>
+    </row>
+    <row r="51" ht="30" customHeight="1" s="235">
+      <c r="A51" s="266" t="n"/>
+      <c r="B51" s="288" t="n"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="266" t="n"/>
+      <c r="B52" s="288" t="n"/>
+      <c r="C52" s="194" t="n"/>
+      <c r="E52" s="182" t="n"/>
+      <c r="F52" s="169" t="n"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="266" t="n"/>
+      <c r="B53" s="288" t="n"/>
+      <c r="E53" s="182" t="n"/>
+    </row>
+    <row r="54">
+      <c r="H54" s="169" t="n"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="248" t="n"/>
+      <c r="B55" s="248" t="n"/>
+      <c r="C55" s="248" t="n"/>
+      <c r="G55" s="169" t="n"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="244" t="n"/>
+      <c r="B56" s="278" t="n"/>
+      <c r="C56" s="295" t="n"/>
+      <c r="G56" s="169" t="n"/>
+    </row>
+    <row r="57">
+      <c r="A57" s="244" t="n"/>
+      <c r="B57" s="282" t="n"/>
+      <c r="C57" s="282" t="n"/>
+      <c r="G57" s="169" t="n"/>
+    </row>
+    <row r="58">
+      <c r="H58" s="169" t="n"/>
+    </row>
+    <row r="59">
+      <c r="H59" s="169" t="n"/>
+    </row>
+    <row r="60">
+      <c r="A60" s="248" t="n"/>
+      <c r="B60" s="248" t="n"/>
+      <c r="H60" s="169" t="n"/>
+    </row>
+    <row r="61">
+      <c r="A61" s="244" t="n"/>
+      <c r="B61" s="295" t="n"/>
+      <c r="H61" s="169" t="n"/>
+    </row>
+    <row r="62">
+      <c r="H62" s="169" t="n"/>
+    </row>
+    <row r="63">
+      <c r="H63" s="169" t="n"/>
+    </row>
+    <row r="64">
+      <c r="H64" s="194" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="13">
+    <mergeCell ref="A28:C28"/>
+    <mergeCell ref="A42:C42"/>
+    <mergeCell ref="A1:J1"/>
+    <mergeCell ref="U1:W1"/>
+    <mergeCell ref="A41:B41"/>
+    <mergeCell ref="A43:B43"/>
+    <mergeCell ref="A31:C31"/>
+    <mergeCell ref="A44:B44"/>
+    <mergeCell ref="A30:C30"/>
+    <mergeCell ref="A39:C39"/>
+    <mergeCell ref="A40:B40"/>
+    <mergeCell ref="A29:C29"/>
+    <mergeCell ref="A6:E6"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr codeName="Sheet4">
+    <tabColor theme="3" tint="-0.499984740745262"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:N39"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="9.140625" defaultRowHeight="15"/>
+  <cols>
+    <col width="3.42578125" customWidth="1" style="3" min="1" max="1"/>
+    <col width="18.42578125" customWidth="1" style="3" min="2" max="2"/>
+    <col width="15.5703125" customWidth="1" style="3" min="3" max="3"/>
+    <col width="21" customWidth="1" style="3" min="4" max="4"/>
+    <col width="23.140625" customWidth="1" style="3" min="5" max="5"/>
+    <col width="20.5703125" customWidth="1" style="3" min="6" max="6"/>
+    <col width="9.28515625" customWidth="1" style="3" min="7" max="7"/>
+    <col width="9.42578125" customWidth="1" style="3" min="8" max="8"/>
+    <col width="13.42578125" bestFit="1" customWidth="1" style="3" min="9" max="10"/>
+    <col width="14.140625" bestFit="1" customWidth="1" style="3" min="11" max="11"/>
+    <col width="9.140625" customWidth="1" style="3" min="12" max="16384"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="D1" s="5" t="n"/>
+      <c r="E1" s="3" t="n"/>
+    </row>
+    <row r="2">
+      <c r="B2" s="248" t="n"/>
+      <c r="C2" s="248" t="n"/>
+      <c r="D2" s="248" t="n"/>
+      <c r="E2" s="248" t="n"/>
+      <c r="F2" s="248" t="n"/>
+    </row>
+    <row r="3">
+      <c r="B3" s="54" t="n"/>
+      <c r="C3" s="200" t="n"/>
+      <c r="D3" s="200" t="n"/>
+      <c r="E3" s="200" t="n"/>
+      <c r="F3" s="21" t="n"/>
+      <c r="G3" s="6" t="n"/>
+      <c r="I3" s="23" t="n"/>
+      <c r="J3" s="70" t="n"/>
+      <c r="K3" s="70" t="n"/>
+      <c r="L3" s="23" t="n"/>
+    </row>
+    <row r="4">
+      <c r="B4" s="54" t="n"/>
+      <c r="C4" s="200" t="n"/>
+      <c r="D4" s="200" t="n"/>
+      <c r="E4" s="200" t="n"/>
+      <c r="F4" s="21" t="n"/>
+      <c r="G4" s="6" t="n"/>
+      <c r="I4" s="23" t="n"/>
+      <c r="J4" s="70" t="n"/>
+      <c r="K4" s="70" t="n"/>
+      <c r="L4" s="23" t="n"/>
+    </row>
+    <row r="5">
+      <c r="B5" s="54" t="n"/>
+      <c r="C5" s="200" t="n"/>
+      <c r="D5" s="200" t="n"/>
+      <c r="E5" s="200" t="n"/>
+      <c r="F5" s="21" t="n"/>
+      <c r="G5" s="6" t="n"/>
+      <c r="I5" s="23" t="n"/>
+      <c r="J5" s="70" t="n"/>
+      <c r="K5" s="70" t="n"/>
+      <c r="L5" s="23" t="n"/>
+    </row>
+    <row r="6">
+      <c r="B6" s="248" t="n"/>
+      <c r="C6" s="284" t="n"/>
+      <c r="D6" s="284" t="n"/>
+      <c r="E6" s="275" t="n"/>
+      <c r="F6" s="86" t="n"/>
+      <c r="J6" s="24" t="n"/>
+    </row>
+    <row r="7">
+      <c r="F7" s="296" t="n"/>
+      <c r="J7" s="24" t="n"/>
+    </row>
+    <row r="8">
+      <c r="J8" s="24" t="n"/>
+    </row>
+    <row r="9"/>
+    <row r="10" ht="15" customHeight="1" s="235">
+      <c r="B10" s="248" t="n"/>
+      <c r="C10" s="248" t="n"/>
+      <c r="D10" s="248" t="n"/>
+      <c r="E10" s="248" t="n"/>
+    </row>
+    <row r="11" ht="15" customHeight="1" s="235">
+      <c r="B11" s="55" t="n"/>
+      <c r="C11" s="68" t="n"/>
+      <c r="D11" s="297" t="n"/>
+      <c r="E11" s="33" t="n"/>
+      <c r="K11" s="3" t="n"/>
+      <c r="N11" s="25" t="n"/>
+    </row>
+    <row r="12" ht="15" customHeight="1" s="235">
+      <c r="B12" s="88" t="n"/>
+      <c r="C12" s="169" t="n"/>
+      <c r="D12" s="298" t="n"/>
+      <c r="E12" s="239" t="n"/>
+      <c r="N12" s="25" t="n"/>
+    </row>
+    <row r="13">
+      <c r="B13" s="6" t="n"/>
+      <c r="D13" s="6" t="n"/>
+    </row>
+    <row r="14" ht="15" customHeight="1" s="235">
+      <c r="B14" s="248" t="n"/>
+      <c r="C14" s="248" t="n"/>
+      <c r="D14" s="248" t="n"/>
+      <c r="E14" s="26" t="n"/>
+    </row>
+    <row r="15" ht="15" customHeight="1" s="235">
+      <c r="B15" s="66" t="n"/>
+      <c r="C15" s="67" t="n"/>
+      <c r="D15" s="27" t="n"/>
+      <c r="E15" s="28" t="n"/>
+      <c r="F15" s="23" t="n"/>
+    </row>
+    <row r="16" ht="15" customHeight="1" s="235">
+      <c r="B16" s="66" t="n"/>
+      <c r="C16" s="67" t="n"/>
+      <c r="D16" s="27" t="n"/>
+      <c r="E16" s="28" t="n"/>
+      <c r="F16" s="23" t="n"/>
+    </row>
+    <row r="17" ht="15" customHeight="1" s="235">
+      <c r="B17" s="66" t="n"/>
+      <c r="C17" s="67" t="n"/>
+      <c r="D17" s="27" t="n"/>
+      <c r="E17" s="28" t="n"/>
+      <c r="F17" s="23" t="n"/>
+    </row>
+    <row r="18" ht="15" customHeight="1" s="235">
+      <c r="B18" s="66" t="n"/>
+      <c r="C18" s="67" t="n"/>
+      <c r="D18" s="27" t="n"/>
+      <c r="E18" s="28" t="n"/>
+      <c r="F18" s="23" t="n"/>
+    </row>
+    <row r="19" ht="15" customHeight="1" s="235">
+      <c r="B19" s="29" t="n"/>
+      <c r="C19" s="206" t="n"/>
+      <c r="D19" s="240" t="n"/>
+      <c r="I19" s="30" t="n"/>
+    </row>
+    <row r="20">
+      <c r="B20" s="6" t="n"/>
+      <c r="C20" s="17" t="n"/>
+      <c r="D20" s="31" t="n"/>
+      <c r="I20" s="30" t="n"/>
+    </row>
+    <row r="21">
+      <c r="B21" s="6" t="n"/>
+      <c r="C21" s="17" t="n"/>
+      <c r="D21" s="31" t="n"/>
+      <c r="I21" s="30" t="n"/>
+    </row>
+    <row r="22"/>
+    <row r="23"/>
+    <row r="24"/>
+    <row r="25" ht="45" customHeight="1" s="235">
+      <c r="B25" s="248" t="n"/>
+      <c r="C25" s="248" t="n"/>
+      <c r="D25" s="248" t="n"/>
+      <c r="E25" s="248" t="n"/>
+      <c r="F25" s="251" t="n"/>
+    </row>
+    <row r="26">
+      <c r="B26" s="172" t="n"/>
+      <c r="C26" s="131" t="n"/>
+      <c r="D26" s="73" t="n"/>
+      <c r="E26" s="200" t="n"/>
+      <c r="F26" s="132" t="n"/>
+    </row>
+    <row r="27">
+      <c r="B27" s="172" t="n"/>
+      <c r="C27" s="131" t="n"/>
+      <c r="D27" s="73" t="n"/>
+      <c r="E27" s="200" t="n"/>
+      <c r="F27" s="132" t="n"/>
+    </row>
+    <row r="28">
+      <c r="B28" s="172" t="n"/>
+      <c r="C28" s="131" t="n"/>
+      <c r="D28" s="73" t="n"/>
+      <c r="E28" s="200" t="n"/>
+      <c r="F28" s="132" t="n"/>
+      <c r="H28" s="3" t="n"/>
+    </row>
+    <row r="29"/>
+    <row r="30"/>
+    <row r="31"/>
+    <row r="32">
+      <c r="B32" s="251" t="n"/>
+      <c r="C32" s="251" t="n"/>
+      <c r="D32" s="251" t="n"/>
+      <c r="E32" s="251" t="n"/>
+    </row>
+    <row r="33">
+      <c r="B33" s="100" t="n"/>
+      <c r="C33" s="263" t="n"/>
+      <c r="D33" s="263" t="n"/>
+      <c r="E33" s="200" t="n"/>
+    </row>
+    <row r="34">
+      <c r="B34" s="100" t="n"/>
+      <c r="C34" s="263" t="n"/>
+      <c r="D34" s="263" t="n"/>
+      <c r="E34" s="200" t="n"/>
+    </row>
+    <row r="35">
+      <c r="B35" s="244" t="n"/>
+      <c r="C35" s="263" t="n"/>
+      <c r="D35" s="263" t="n"/>
+      <c r="E35" s="200" t="n"/>
+    </row>
+    <row r="36">
+      <c r="B36" s="100" t="n"/>
+      <c r="C36" s="263" t="n"/>
+      <c r="D36" s="263" t="n"/>
+      <c r="E36" s="200" t="n"/>
+    </row>
+    <row r="37">
+      <c r="B37" s="244" t="n"/>
+      <c r="C37" s="263" t="n"/>
+      <c r="D37" s="263" t="n"/>
+      <c r="E37" s="200" t="n"/>
+    </row>
+    <row r="38">
+      <c r="B38" s="244" t="n"/>
+      <c r="C38" s="263" t="n"/>
+      <c r="D38" s="263" t="n"/>
+      <c r="E38" s="200" t="n"/>
+    </row>
+    <row r="39">
+      <c r="B39" s="244" t="n"/>
+      <c r="C39" s="263" t="n"/>
+      <c r="D39" s="263" t="n"/>
+      <c r="E39" s="200" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="B6:E6"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr codeName="Sheet5">
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:L23"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="9.140625" defaultRowHeight="15"/>
+  <cols>
+    <col width="2.7109375" customWidth="1" style="235" min="1" max="1"/>
+    <col width="12.7109375" customWidth="1" style="235" min="2" max="2"/>
+    <col width="15.7109375" customWidth="1" style="235" min="3" max="3"/>
+    <col width="21.85546875" customWidth="1" style="235" min="4" max="4"/>
+    <col width="22.28515625" customWidth="1" style="235" min="5" max="5"/>
+    <col width="19.7109375" customWidth="1" style="235" min="6" max="6"/>
+    <col width="9.140625" customWidth="1" style="235" min="7" max="7"/>
+    <col width="12" customWidth="1" style="235" min="8" max="8"/>
+    <col width="12.42578125" bestFit="1" customWidth="1" style="235" min="9" max="9"/>
+    <col width="9.42578125" bestFit="1" customWidth="1" style="235" min="10" max="10"/>
+    <col width="13.42578125" bestFit="1" customWidth="1" style="235" min="11" max="11"/>
+    <col width="10" bestFit="1" customWidth="1" style="235" min="12" max="12"/>
+    <col width="9.140625" customWidth="1" style="235" min="13" max="16384"/>
+  </cols>
+  <sheetData>
+    <row r="1"/>
+    <row r="2">
+      <c r="B2" s="248" t="n"/>
+      <c r="C2" s="248" t="n"/>
+      <c r="D2" s="248" t="n"/>
+      <c r="E2" s="248" t="n"/>
+      <c r="F2" s="248" t="n"/>
+      <c r="J2" s="194" t="n"/>
+    </row>
+    <row r="3">
+      <c r="B3" s="54" t="n"/>
+      <c r="C3" s="295" t="n"/>
+      <c r="D3" s="200" t="n"/>
+      <c r="E3" s="200" t="n"/>
+      <c r="F3" s="21" t="n"/>
+      <c r="G3" s="6" t="n"/>
+      <c r="H3" s="257" t="n"/>
+      <c r="I3" s="278" t="n"/>
+      <c r="J3" s="194" t="n"/>
+      <c r="K3" s="278" t="n"/>
+      <c r="L3" s="278" t="n"/>
+    </row>
+    <row r="4">
+      <c r="B4" s="54" t="n"/>
+      <c r="C4" s="295" t="n"/>
+      <c r="D4" s="200" t="n"/>
+      <c r="E4" s="200" t="n"/>
+      <c r="F4" s="21" t="n"/>
+      <c r="G4" s="6" t="n"/>
+      <c r="H4" s="257" t="n"/>
+      <c r="I4" s="278" t="n"/>
+      <c r="J4" s="194" t="n"/>
+      <c r="K4" s="278" t="n"/>
+      <c r="L4" s="278" t="n"/>
+    </row>
+    <row r="5">
+      <c r="B5" s="54" t="n"/>
+      <c r="C5" s="295" t="n"/>
+      <c r="D5" s="200" t="n"/>
+      <c r="E5" s="200" t="n"/>
+      <c r="F5" s="21" t="n"/>
+      <c r="G5" s="6" t="n"/>
+      <c r="H5" s="257" t="n"/>
+      <c r="I5" s="278" t="n"/>
+      <c r="J5" s="194" t="n"/>
+      <c r="K5" s="278" t="n"/>
+      <c r="L5" s="278" t="n"/>
+    </row>
+    <row r="6">
+      <c r="B6" s="248" t="n"/>
+      <c r="C6" s="284" t="n"/>
+      <c r="D6" s="284" t="n"/>
+      <c r="E6" s="275" t="n"/>
+      <c r="F6" s="86" t="n"/>
+      <c r="H6" s="278" t="n"/>
+      <c r="I6" s="194" t="n"/>
+      <c r="J6" s="194" t="n"/>
+    </row>
+    <row r="7">
+      <c r="B7" s="299" t="n"/>
+      <c r="C7" s="299" t="n"/>
+      <c r="D7" s="299" t="n"/>
+      <c r="E7" s="299" t="n"/>
+      <c r="F7" s="300" t="n"/>
+      <c r="I7" s="194" t="n"/>
+      <c r="J7" s="194" t="n"/>
+    </row>
+    <row r="8">
+      <c r="B8" s="299" t="n"/>
+      <c r="C8" s="299" t="n"/>
+      <c r="D8" s="299" t="n"/>
+      <c r="E8" s="299" t="n"/>
+      <c r="F8" s="300" t="n"/>
+    </row>
+    <row r="9">
+      <c r="B9" s="248" t="n"/>
+      <c r="C9" s="248" t="n"/>
+      <c r="D9" s="248" t="n"/>
+      <c r="E9" s="248" t="n"/>
+      <c r="F9" s="299" t="n"/>
+    </row>
+    <row r="10">
+      <c r="B10" s="55" t="n"/>
+      <c r="C10" s="68" t="n"/>
+      <c r="D10" s="68" t="n"/>
+      <c r="E10" s="301" t="n"/>
+      <c r="F10" s="299" t="n"/>
+    </row>
+    <row r="11"/>
+    <row r="12" ht="30" customHeight="1" s="235">
+      <c r="B12" s="248" t="n"/>
+      <c r="C12" s="248" t="n"/>
+      <c r="D12" s="248" t="n"/>
+      <c r="E12" s="248" t="n"/>
+      <c r="F12" s="251" t="n"/>
+    </row>
+    <row r="13">
+      <c r="B13" s="172" t="n"/>
+      <c r="C13" s="302" t="n"/>
+      <c r="D13" s="73" t="n"/>
+      <c r="E13" s="68" t="n"/>
+      <c r="F13" s="132" t="n"/>
+    </row>
+    <row r="14">
+      <c r="B14" s="172" t="n"/>
+      <c r="C14" s="303" t="n"/>
+      <c r="D14" s="73" t="n"/>
+      <c r="E14" s="68" t="n"/>
+      <c r="F14" s="132" t="n"/>
+    </row>
+    <row r="15">
+      <c r="B15" s="172" t="n"/>
+      <c r="C15" s="166" t="n"/>
+      <c r="D15" s="171" t="n"/>
+      <c r="E15" s="68" t="n"/>
+      <c r="F15" s="132" t="n"/>
+    </row>
+    <row r="16"/>
+    <row r="17"/>
+    <row r="18"/>
+    <row r="19" ht="30" customHeight="1" s="235">
+      <c r="C19" s="248" t="n"/>
+      <c r="D19" s="248" t="n"/>
+      <c r="E19" s="248" t="n"/>
+    </row>
+    <row r="20">
+      <c r="C20" s="244" t="n"/>
+      <c r="D20" s="68" t="n"/>
+      <c r="E20" s="191" t="n"/>
+    </row>
+    <row r="21">
+      <c r="C21" s="244" t="n"/>
+      <c r="D21" s="68" t="n"/>
+      <c r="E21" s="191" t="n"/>
+    </row>
+    <row r="22">
+      <c r="C22" s="244" t="n"/>
+      <c r="D22" s="68" t="n"/>
+      <c r="E22" s="191" t="n"/>
+    </row>
+    <row r="23">
+      <c r="D23" s="169" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="C13:C15"/>
+    <mergeCell ref="B6:E6"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr codeName="Sheet8">
+    <tabColor theme="3" tint="-0.499984740745262"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J12"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="13" defaultRowHeight="15"/>
+  <cols>
+    <col width="9.5703125" bestFit="1" customWidth="1" style="235" min="1" max="1"/>
+    <col width="13" customWidth="1" style="235" min="2" max="2"/>
+    <col width="11.140625" customWidth="1" style="235" min="3" max="3"/>
+    <col width="14.28515625" bestFit="1" customWidth="1" style="235" min="4" max="4"/>
+    <col width="20.85546875" customWidth="1" style="235" min="5" max="5"/>
+    <col width="7.5703125" customWidth="1" style="235" min="6" max="6"/>
+    <col width="11.5703125" customWidth="1" style="235" min="7" max="7"/>
+    <col width="14.28515625" customWidth="1" style="235" min="8" max="8"/>
+    <col width="14.28515625" bestFit="1" customWidth="1" style="235" min="9" max="9"/>
+    <col width="13" customWidth="1" style="235" min="10" max="16384"/>
+  </cols>
+  <sheetData>
+    <row r="1"/>
+    <row r="2">
+      <c r="B2" s="248" t="n"/>
+      <c r="C2" s="284" t="n"/>
+      <c r="D2" s="284" t="n"/>
+      <c r="E2" s="284" t="n"/>
+      <c r="F2" s="284" t="n"/>
+      <c r="G2" s="284" t="n"/>
+      <c r="H2" s="284" t="n"/>
+      <c r="I2" s="275" t="n"/>
+    </row>
+    <row r="3" ht="30" customHeight="1" s="235">
+      <c r="B3" s="248" t="n"/>
+      <c r="C3" s="248" t="n"/>
+      <c r="D3" s="248" t="n"/>
+      <c r="E3" s="248" t="n"/>
+      <c r="F3" s="248" t="n"/>
+      <c r="G3" s="248" t="n"/>
+      <c r="H3" s="248" t="n"/>
+      <c r="I3" s="248" t="n"/>
+    </row>
+    <row r="4">
+      <c r="B4" s="48" t="n"/>
+      <c r="C4" s="76" t="n"/>
+      <c r="D4" s="100" t="n"/>
+      <c r="E4" s="181" t="n"/>
+      <c r="F4" s="295" t="n"/>
+      <c r="G4" s="295" t="n"/>
+      <c r="H4" s="295" t="n"/>
+      <c r="I4" s="288" t="n"/>
+    </row>
+    <row r="5">
+      <c r="B5" s="48" t="n"/>
+      <c r="C5" s="76" t="n"/>
+      <c r="D5" s="100" t="n"/>
+      <c r="E5" s="181" t="n"/>
+      <c r="F5" s="295" t="n"/>
+      <c r="G5" s="295" t="n"/>
+      <c r="H5" s="295" t="n"/>
+      <c r="I5" s="288" t="n"/>
+    </row>
+    <row r="6">
+      <c r="B6" s="48" t="n"/>
+      <c r="C6" s="76" t="n"/>
+      <c r="D6" s="244" t="n"/>
+      <c r="E6" s="181" t="n"/>
+      <c r="F6" s="295" t="n"/>
+      <c r="G6" s="295" t="n"/>
+      <c r="H6" s="295" t="n"/>
+      <c r="I6" s="288" t="n"/>
+    </row>
+    <row r="7">
+      <c r="B7" s="45" t="n"/>
+      <c r="C7" s="46" t="n"/>
+      <c r="D7" s="45" t="n"/>
+      <c r="F7" s="299" t="n"/>
+    </row>
+    <row r="8">
+      <c r="B8" s="248" t="n"/>
+      <c r="C8" s="284" t="n"/>
+      <c r="D8" s="284" t="n"/>
+      <c r="E8" s="284" t="n"/>
+      <c r="F8" s="284" t="n"/>
+      <c r="G8" s="284" t="n"/>
+      <c r="H8" s="284" t="n"/>
+      <c r="I8" s="275" t="n"/>
+    </row>
+    <row r="9" ht="30" customHeight="1" s="235">
+      <c r="B9" s="248" t="n"/>
+      <c r="C9" s="248" t="n"/>
+      <c r="D9" s="248" t="n"/>
+      <c r="E9" s="248" t="n"/>
+      <c r="F9" s="248" t="n"/>
+      <c r="G9" s="248" t="n"/>
+      <c r="H9" s="248" t="n"/>
+      <c r="I9" s="248" t="n"/>
+    </row>
+    <row r="10">
+      <c r="B10" s="48" t="n"/>
+      <c r="C10" s="76" t="n"/>
+      <c r="D10" s="100" t="n"/>
+      <c r="E10" s="48" t="n"/>
+      <c r="F10" s="295" t="n"/>
+      <c r="G10" s="295" t="n"/>
+      <c r="H10" s="295" t="n"/>
+      <c r="I10" s="288" t="n"/>
+      <c r="J10" s="299" t="n"/>
+    </row>
+    <row r="11">
+      <c r="B11" s="48" t="n"/>
+      <c r="C11" s="76" t="n"/>
+      <c r="D11" s="72" t="n"/>
+      <c r="E11" s="48" t="n"/>
+      <c r="F11" s="295" t="n"/>
+      <c r="G11" s="295" t="n"/>
+      <c r="H11" s="295" t="n"/>
+      <c r="I11" s="288" t="n"/>
+      <c r="J11" s="299" t="n"/>
+    </row>
+    <row r="12">
+      <c r="B12" s="48" t="n"/>
+      <c r="C12" s="76" t="n"/>
+      <c r="D12" s="72" t="n"/>
+      <c r="E12" s="48" t="n"/>
+      <c r="F12" s="295" t="n"/>
+      <c r="G12" s="295" t="n"/>
+      <c r="H12" s="295" t="n"/>
+      <c r="I12" s="288" t="n"/>
+      <c r="J12" s="299" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="B8:I8"/>
+    <mergeCell ref="B2:I2"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr codeName="Sheet6">
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
@@ -2262,11 +4044,11 @@
     <row r="1"/>
     <row r="2" ht="15" customHeight="1" s="235">
       <c r="B2" s="248" t="n"/>
-      <c r="C2" s="275" t="n"/>
-      <c r="D2" s="276" t="n"/>
+      <c r="C2" s="284" t="n"/>
+      <c r="D2" s="275" t="n"/>
       <c r="F2" s="248" t="n"/>
-      <c r="G2" s="275" t="n"/>
-      <c r="H2" s="276" t="n"/>
+      <c r="G2" s="284" t="n"/>
+      <c r="H2" s="275" t="n"/>
     </row>
     <row r="3" ht="15" customHeight="1" s="235">
       <c r="B3" s="248" t="n"/>
@@ -2278,8 +4060,8 @@
     </row>
     <row r="4">
       <c r="B4" s="22" t="n"/>
-      <c r="C4" s="277" t="n"/>
-      <c r="D4" s="277" t="n"/>
+      <c r="C4" s="304" t="n"/>
+      <c r="D4" s="304" t="n"/>
       <c r="F4" s="22" t="n"/>
       <c r="G4" s="32" t="n"/>
       <c r="H4" s="32" t="n"/>
@@ -2287,59 +4069,59 @@
     </row>
     <row r="5" customFormat="1" s="5">
       <c r="B5" s="248" t="n"/>
-      <c r="C5" s="278" t="n"/>
-      <c r="D5" s="278" t="n"/>
-      <c r="E5" s="279" t="n"/>
+      <c r="C5" s="305" t="n"/>
+      <c r="D5" s="305" t="n"/>
+      <c r="E5" s="306" t="n"/>
       <c r="F5" s="248" t="n"/>
-      <c r="G5" s="278" t="n"/>
-      <c r="H5" s="278" t="n"/>
+      <c r="G5" s="305" t="n"/>
+      <c r="H5" s="305" t="n"/>
       <c r="J5" s="8" t="n"/>
     </row>
     <row r="6" customFormat="1" s="5">
       <c r="C6" s="3" t="n"/>
       <c r="D6" s="3" t="n"/>
-      <c r="E6" s="279" t="n"/>
+      <c r="E6" s="306" t="n"/>
     </row>
     <row r="7" customFormat="1" s="5">
       <c r="B7" s="3" t="n"/>
       <c r="C7" s="3" t="n"/>
       <c r="D7" s="3" t="n"/>
-      <c r="E7" s="279" t="n"/>
+      <c r="E7" s="306" t="n"/>
     </row>
     <row r="8">
       <c r="B8" s="98" t="n"/>
     </row>
     <row r="9">
-      <c r="B9" s="280" t="n"/>
-      <c r="C9" s="280" t="n"/>
+      <c r="B9" s="307" t="n"/>
+      <c r="C9" s="307" t="n"/>
     </row>
     <row r="10">
       <c r="B10" s="281" t="n"/>
-      <c r="C10" s="282" t="n"/>
+      <c r="C10" s="288" t="n"/>
     </row>
     <row r="11">
       <c r="B11" s="281" t="n"/>
-      <c r="C11" s="282" t="n"/>
+      <c r="C11" s="288" t="n"/>
     </row>
     <row r="12">
       <c r="B12" s="281" t="n"/>
-      <c r="C12" s="282" t="n"/>
+      <c r="C12" s="288" t="n"/>
     </row>
     <row r="13">
       <c r="B13" s="281" t="n"/>
-      <c r="C13" s="283" t="n"/>
+      <c r="C13" s="308" t="n"/>
     </row>
     <row r="14">
       <c r="B14" s="281" t="n"/>
-      <c r="C14" s="283" t="n"/>
+      <c r="C14" s="308" t="n"/>
     </row>
     <row r="15">
       <c r="B15" s="281" t="n"/>
-      <c r="C15" s="283" t="n"/>
+      <c r="C15" s="308" t="n"/>
     </row>
     <row r="16">
       <c r="B16" s="281" t="n"/>
-      <c r="C16" s="283" t="n"/>
+      <c r="C16" s="308" t="n"/>
     </row>
     <row r="17">
       <c r="B17" s="281" t="n"/>
@@ -2351,19 +4133,19 @@
     </row>
     <row r="19">
       <c r="B19" s="281" t="n"/>
-      <c r="C19" s="282" t="n"/>
+      <c r="C19" s="288" t="n"/>
     </row>
     <row r="20">
       <c r="B20" s="281" t="n"/>
-      <c r="C20" s="282" t="n"/>
+      <c r="C20" s="288" t="n"/>
     </row>
     <row r="21">
       <c r="B21" s="281" t="n"/>
-      <c r="C21" s="282" t="n"/>
+      <c r="C21" s="288" t="n"/>
     </row>
     <row r="22">
       <c r="B22" s="181" t="n"/>
-      <c r="C22" s="284" t="n"/>
+      <c r="C22" s="309" t="n"/>
     </row>
     <row r="23"/>
     <row r="24"/>
@@ -2382,7 +4164,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr codeName="Sheet9">
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2408,180 +4190,180 @@
   <sheetData>
     <row r="1">
       <c r="B1" s="266" t="n"/>
-      <c r="C1" s="275" t="n"/>
-      <c r="D1" s="276" t="n"/>
+      <c r="C1" s="284" t="n"/>
+      <c r="D1" s="275" t="n"/>
       <c r="E1" s="266" t="n"/>
-      <c r="F1" s="276" t="n"/>
+      <c r="F1" s="275" t="n"/>
       <c r="H1" s="266" t="n"/>
-      <c r="I1" s="275" t="n"/>
-      <c r="J1" s="276" t="n"/>
+      <c r="I1" s="284" t="n"/>
+      <c r="J1" s="275" t="n"/>
       <c r="K1" s="266" t="n"/>
-      <c r="L1" s="276" t="n"/>
+      <c r="L1" s="275" t="n"/>
     </row>
     <row r="2">
       <c r="B2" s="266" t="n"/>
-      <c r="C2" s="275" t="n"/>
-      <c r="D2" s="276" t="n"/>
+      <c r="C2" s="284" t="n"/>
+      <c r="D2" s="275" t="n"/>
       <c r="E2" s="266" t="n"/>
-      <c r="F2" s="276" t="n"/>
+      <c r="F2" s="275" t="n"/>
       <c r="H2" s="266" t="n"/>
-      <c r="I2" s="275" t="n"/>
-      <c r="J2" s="276" t="n"/>
+      <c r="I2" s="284" t="n"/>
+      <c r="J2" s="275" t="n"/>
       <c r="K2" s="266" t="n"/>
-      <c r="L2" s="276" t="n"/>
+      <c r="L2" s="275" t="n"/>
     </row>
     <row r="3">
       <c r="B3" s="266" t="n"/>
-      <c r="C3" s="275" t="n"/>
-      <c r="D3" s="275" t="n"/>
-      <c r="E3" s="275" t="n"/>
-      <c r="F3" s="276" t="n"/>
+      <c r="C3" s="284" t="n"/>
+      <c r="D3" s="284" t="n"/>
+      <c r="E3" s="284" t="n"/>
+      <c r="F3" s="275" t="n"/>
       <c r="H3" s="266" t="n"/>
-      <c r="I3" s="275" t="n"/>
-      <c r="J3" s="275" t="n"/>
-      <c r="K3" s="275" t="n"/>
-      <c r="L3" s="276" t="n"/>
+      <c r="I3" s="284" t="n"/>
+      <c r="J3" s="284" t="n"/>
+      <c r="K3" s="284" t="n"/>
+      <c r="L3" s="275" t="n"/>
     </row>
     <row r="4">
       <c r="B4" s="263" t="n"/>
       <c r="C4" s="263" t="n"/>
       <c r="D4" s="263" t="n"/>
-      <c r="E4" s="276" t="n"/>
+      <c r="E4" s="275" t="n"/>
       <c r="F4" s="263" t="n"/>
       <c r="H4" s="263" t="n"/>
       <c r="I4" s="263" t="n"/>
       <c r="J4" s="263" t="n"/>
-      <c r="K4" s="276" t="n"/>
+      <c r="K4" s="275" t="n"/>
       <c r="L4" s="263" t="n"/>
     </row>
     <row r="5" ht="15" customHeight="1" s="235">
       <c r="B5" s="237" t="n"/>
       <c r="C5" s="266" t="n"/>
-      <c r="D5" s="285" t="n"/>
-      <c r="E5" s="276" t="n"/>
-      <c r="F5" s="286" t="n"/>
+      <c r="D5" s="310" t="n"/>
+      <c r="E5" s="275" t="n"/>
+      <c r="F5" s="311" t="n"/>
       <c r="H5" s="237" t="n"/>
       <c r="I5" s="266" t="n"/>
-      <c r="J5" s="285" t="n"/>
-      <c r="K5" s="276" t="n"/>
-      <c r="L5" s="286" t="n"/>
+      <c r="J5" s="310" t="n"/>
+      <c r="K5" s="275" t="n"/>
+      <c r="L5" s="311" t="n"/>
     </row>
     <row r="6">
-      <c r="B6" s="287" t="n"/>
+      <c r="B6" s="303" t="n"/>
       <c r="C6" s="266" t="n"/>
-      <c r="D6" s="285" t="n"/>
-      <c r="E6" s="276" t="n"/>
-      <c r="F6" s="287" t="n"/>
-      <c r="H6" s="287" t="n"/>
+      <c r="D6" s="310" t="n"/>
+      <c r="E6" s="275" t="n"/>
+      <c r="F6" s="303" t="n"/>
+      <c r="H6" s="303" t="n"/>
       <c r="I6" s="266" t="n"/>
-      <c r="J6" s="285" t="n"/>
-      <c r="K6" s="276" t="n"/>
-      <c r="L6" s="287" t="n"/>
+      <c r="J6" s="310" t="n"/>
+      <c r="K6" s="275" t="n"/>
+      <c r="L6" s="303" t="n"/>
     </row>
     <row r="7">
-      <c r="B7" s="287" t="n"/>
+      <c r="B7" s="303" t="n"/>
       <c r="C7" s="266" t="n"/>
-      <c r="D7" s="285" t="n"/>
-      <c r="E7" s="276" t="n"/>
-      <c r="F7" s="287" t="n"/>
-      <c r="H7" s="287" t="n"/>
+      <c r="D7" s="310" t="n"/>
+      <c r="E7" s="275" t="n"/>
+      <c r="F7" s="303" t="n"/>
+      <c r="H7" s="303" t="n"/>
       <c r="I7" s="266" t="n"/>
-      <c r="J7" s="285" t="n"/>
-      <c r="K7" s="276" t="n"/>
-      <c r="L7" s="287" t="n"/>
+      <c r="J7" s="310" t="n"/>
+      <c r="K7" s="275" t="n"/>
+      <c r="L7" s="303" t="n"/>
     </row>
     <row r="8">
-      <c r="B8" s="287" t="n"/>
+      <c r="B8" s="303" t="n"/>
       <c r="C8" s="266" t="n"/>
-      <c r="D8" s="285" t="n"/>
-      <c r="E8" s="276" t="n"/>
-      <c r="F8" s="287" t="n"/>
-      <c r="H8" s="287" t="n"/>
+      <c r="D8" s="310" t="n"/>
+      <c r="E8" s="275" t="n"/>
+      <c r="F8" s="303" t="n"/>
+      <c r="H8" s="303" t="n"/>
       <c r="I8" s="266" t="n"/>
-      <c r="J8" s="285" t="n"/>
-      <c r="K8" s="276" t="n"/>
-      <c r="L8" s="287" t="n"/>
+      <c r="J8" s="310" t="n"/>
+      <c r="K8" s="275" t="n"/>
+      <c r="L8" s="303" t="n"/>
     </row>
     <row r="9">
       <c r="B9" s="166" t="n"/>
       <c r="C9" s="266" t="n"/>
-      <c r="D9" s="285" t="n"/>
-      <c r="E9" s="276" t="n"/>
+      <c r="D9" s="310" t="n"/>
+      <c r="E9" s="275" t="n"/>
       <c r="F9" s="166" t="n"/>
       <c r="H9" s="166" t="n"/>
       <c r="I9" s="266" t="n"/>
-      <c r="J9" s="285" t="n"/>
-      <c r="K9" s="276" t="n"/>
+      <c r="J9" s="310" t="n"/>
+      <c r="K9" s="275" t="n"/>
       <c r="L9" s="166" t="n"/>
     </row>
     <row r="10">
       <c r="B10" s="233" t="n"/>
       <c r="C10" s="230" t="n"/>
-      <c r="D10" s="288" t="n"/>
-      <c r="E10" s="288" t="n"/>
+      <c r="D10" s="312" t="n"/>
+      <c r="E10" s="312" t="n"/>
       <c r="I10" s="230" t="n"/>
-      <c r="J10" s="288" t="n"/>
-      <c r="K10" s="288" t="n"/>
+      <c r="J10" s="312" t="n"/>
+      <c r="K10" s="312" t="n"/>
     </row>
     <row r="11"/>
     <row r="12" ht="15" customHeight="1" s="235">
       <c r="B12" s="266" t="n"/>
-      <c r="C12" s="275" t="n"/>
-      <c r="D12" s="276" t="n"/>
+      <c r="C12" s="284" t="n"/>
+      <c r="D12" s="275" t="n"/>
       <c r="E12" s="266" t="n"/>
-      <c r="F12" s="276" t="n"/>
+      <c r="F12" s="275" t="n"/>
       <c r="H12" s="266" t="n"/>
-      <c r="I12" s="275" t="n"/>
-      <c r="J12" s="276" t="n"/>
+      <c r="I12" s="284" t="n"/>
+      <c r="J12" s="275" t="n"/>
       <c r="K12" s="266" t="n"/>
-      <c r="L12" s="276" t="n"/>
+      <c r="L12" s="275" t="n"/>
     </row>
     <row r="13" ht="15" customHeight="1" s="235">
       <c r="B13" s="266" t="n"/>
-      <c r="C13" s="275" t="n"/>
-      <c r="D13" s="276" t="n"/>
+      <c r="C13" s="284" t="n"/>
+      <c r="D13" s="275" t="n"/>
       <c r="E13" s="266" t="n"/>
-      <c r="F13" s="276" t="n"/>
+      <c r="F13" s="275" t="n"/>
       <c r="H13" s="266" t="n"/>
-      <c r="I13" s="275" t="n"/>
-      <c r="J13" s="276" t="n"/>
+      <c r="I13" s="284" t="n"/>
+      <c r="J13" s="275" t="n"/>
       <c r="K13" s="266" t="n"/>
-      <c r="L13" s="276" t="n"/>
+      <c r="L13" s="275" t="n"/>
     </row>
     <row r="14" ht="15" customHeight="1" s="235">
       <c r="B14" s="266" t="n"/>
-      <c r="C14" s="275" t="n"/>
-      <c r="D14" s="275" t="n"/>
-      <c r="E14" s="275" t="n"/>
-      <c r="F14" s="276" t="n"/>
+      <c r="C14" s="284" t="n"/>
+      <c r="D14" s="284" t="n"/>
+      <c r="E14" s="284" t="n"/>
+      <c r="F14" s="275" t="n"/>
       <c r="H14" s="266" t="n"/>
-      <c r="I14" s="275" t="n"/>
-      <c r="J14" s="275" t="n"/>
-      <c r="K14" s="275" t="n"/>
-      <c r="L14" s="276" t="n"/>
+      <c r="I14" s="284" t="n"/>
+      <c r="J14" s="284" t="n"/>
+      <c r="K14" s="284" t="n"/>
+      <c r="L14" s="275" t="n"/>
     </row>
     <row r="15">
       <c r="B15" s="263" t="n"/>
       <c r="C15" s="263" t="n"/>
       <c r="D15" s="263" t="n"/>
-      <c r="E15" s="276" t="n"/>
+      <c r="E15" s="275" t="n"/>
       <c r="F15" s="263" t="n"/>
       <c r="H15" s="263" t="n"/>
       <c r="I15" s="263" t="n"/>
       <c r="J15" s="263" t="n"/>
-      <c r="K15" s="276" t="n"/>
+      <c r="K15" s="275" t="n"/>
       <c r="L15" s="263" t="n"/>
     </row>
     <row r="16" ht="15" customHeight="1" s="235">
       <c r="B16" s="237" t="n"/>
       <c r="C16" s="266" t="n"/>
-      <c r="D16" s="285" t="n"/>
-      <c r="E16" s="276" t="n"/>
+      <c r="D16" s="310" t="n"/>
+      <c r="E16" s="275" t="n"/>
       <c r="F16" s="232" t="n"/>
       <c r="H16" s="237" t="n"/>
       <c r="I16" s="266" t="n"/>
-      <c r="J16" s="285" t="n"/>
-      <c r="K16" s="276" t="n"/>
+      <c r="J16" s="310" t="n"/>
+      <c r="K16" s="275" t="n"/>
       <c r="L16" s="232" t="n"/>
     </row>
     <row r="17"/>
@@ -2711,7 +4493,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr codeName="Sheet7">
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2738,10 +4520,10 @@
   <sheetData>
     <row r="1" ht="15.75" customHeight="1" s="235">
       <c r="B1" s="274" t="n"/>
-      <c r="C1" s="275" t="n"/>
-      <c r="D1" s="275" t="n"/>
-      <c r="E1" s="275" t="n"/>
-      <c r="F1" s="276" t="n"/>
+      <c r="C1" s="284" t="n"/>
+      <c r="D1" s="284" t="n"/>
+      <c r="E1" s="284" t="n"/>
+      <c r="F1" s="275" t="n"/>
     </row>
     <row r="2" ht="15" customHeight="1" s="235">
       <c r="B2" s="274" t="n"/>
@@ -2763,7 +4545,7 @@
       <c r="F3" s="221" t="n"/>
       <c r="J3" s="81" t="n"/>
       <c r="K3" s="56" t="n"/>
-      <c r="L3" s="289" t="n"/>
+      <c r="L3" s="313" t="n"/>
       <c r="M3" s="57" t="n"/>
       <c r="N3" s="53" t="n"/>
     </row>
@@ -2775,7 +4557,7 @@
       <c r="F4" s="221" t="n"/>
       <c r="J4" s="81" t="n"/>
       <c r="K4" s="56" t="n"/>
-      <c r="L4" s="289" t="n"/>
+      <c r="L4" s="313" t="n"/>
       <c r="M4" s="57" t="n"/>
       <c r="N4" s="53" t="n"/>
     </row>
@@ -2787,7 +4569,7 @@
       <c r="F5" s="221" t="n"/>
       <c r="J5" s="81" t="n"/>
       <c r="K5" s="56" t="n"/>
-      <c r="L5" s="283" t="n"/>
+      <c r="L5" s="308" t="n"/>
       <c r="M5" s="57" t="n"/>
       <c r="N5" s="53" t="n"/>
     </row>
@@ -2799,7 +4581,7 @@
       <c r="F6" s="221" t="n"/>
       <c r="J6" s="81" t="n"/>
       <c r="K6" s="56" t="n"/>
-      <c r="L6" s="283" t="n"/>
+      <c r="L6" s="308" t="n"/>
       <c r="M6" s="57" t="n"/>
       <c r="N6" s="53" t="n"/>
     </row>
@@ -2811,7 +4593,7 @@
       <c r="F7" s="221" t="n"/>
       <c r="J7" s="81" t="n"/>
       <c r="K7" s="56" t="n"/>
-      <c r="L7" s="283" t="n"/>
+      <c r="L7" s="308" t="n"/>
       <c r="M7" s="57" t="n"/>
       <c r="N7" s="53" t="n"/>
     </row>
@@ -2823,7 +4605,7 @@
       <c r="F8" s="221" t="n"/>
       <c r="J8" s="81" t="n"/>
       <c r="K8" s="140" t="n"/>
-      <c r="L8" s="283" t="n"/>
+      <c r="L8" s="308" t="n"/>
       <c r="M8" s="57" t="n"/>
       <c r="N8" s="53" t="n"/>
     </row>
@@ -2851,89 +4633,89 @@
     <row r="11" ht="15" customFormat="1" customHeight="1" s="184">
       <c r="B11" s="81" t="n"/>
       <c r="C11" s="56" t="n"/>
-      <c r="D11" s="290" t="n"/>
+      <c r="D11" s="314" t="n"/>
       <c r="E11" s="185" t="n"/>
       <c r="F11" s="53" t="n"/>
       <c r="I11" s="177" t="n"/>
       <c r="J11" s="81" t="n"/>
       <c r="K11" s="56" t="n"/>
-      <c r="L11" s="290" t="n"/>
+      <c r="L11" s="314" t="n"/>
       <c r="M11" s="185" t="n"/>
       <c r="N11" s="53" t="n"/>
     </row>
     <row r="12" ht="15" customFormat="1" customHeight="1" s="184">
       <c r="B12" s="81" t="n"/>
       <c r="C12" s="56" t="n"/>
-      <c r="D12" s="290" t="n"/>
+      <c r="D12" s="314" t="n"/>
       <c r="E12" s="185" t="n"/>
       <c r="F12" s="53" t="n"/>
       <c r="I12" s="177" t="n"/>
       <c r="J12" s="81" t="n"/>
       <c r="K12" s="56" t="n"/>
-      <c r="L12" s="290" t="n"/>
+      <c r="L12" s="314" t="n"/>
       <c r="M12" s="185" t="n"/>
       <c r="N12" s="53" t="n"/>
     </row>
     <row r="13" ht="15" customFormat="1" customHeight="1" s="184">
       <c r="B13" s="81" t="n"/>
       <c r="C13" s="56" t="n"/>
-      <c r="D13" s="290" t="n"/>
+      <c r="D13" s="314" t="n"/>
       <c r="E13" s="185" t="n"/>
       <c r="F13" s="53" t="n"/>
       <c r="I13" s="177" t="n"/>
       <c r="J13" s="81" t="n"/>
       <c r="K13" s="56" t="n"/>
-      <c r="L13" s="291" t="n"/>
+      <c r="L13" s="299" t="n"/>
       <c r="M13" s="185" t="n"/>
       <c r="N13" s="53" t="n"/>
     </row>
     <row r="14" ht="15" customFormat="1" customHeight="1" s="184">
       <c r="B14" s="81" t="n"/>
       <c r="C14" s="56" t="n"/>
-      <c r="D14" s="290" t="n"/>
+      <c r="D14" s="314" t="n"/>
       <c r="E14" s="185" t="n"/>
       <c r="F14" s="53" t="n"/>
       <c r="I14" s="177" t="n"/>
       <c r="J14" s="81" t="n"/>
       <c r="K14" s="56" t="n"/>
-      <c r="L14" s="290" t="n"/>
+      <c r="L14" s="314" t="n"/>
       <c r="M14" s="185" t="n"/>
       <c r="N14" s="53" t="n"/>
     </row>
     <row r="15" ht="15" customHeight="1" s="235">
       <c r="B15" s="81" t="n"/>
       <c r="C15" s="56" t="n"/>
-      <c r="D15" s="291" t="n"/>
+      <c r="D15" s="299" t="n"/>
       <c r="E15" s="185" t="n"/>
       <c r="F15" s="53" t="n"/>
       <c r="I15" s="177" t="n"/>
       <c r="J15" s="81" t="n"/>
       <c r="K15" s="56" t="n"/>
-      <c r="L15" s="290" t="n"/>
+      <c r="L15" s="314" t="n"/>
       <c r="M15" s="185" t="n"/>
       <c r="N15" s="53" t="n"/>
     </row>
     <row r="16" ht="15" customHeight="1" s="235">
       <c r="B16" s="81" t="n"/>
       <c r="C16" s="56" t="n"/>
-      <c r="D16" s="290" t="n"/>
+      <c r="D16" s="314" t="n"/>
       <c r="E16" s="185" t="n"/>
       <c r="F16" s="53" t="n"/>
       <c r="J16" s="81" t="n"/>
       <c r="K16" s="56" t="n"/>
-      <c r="L16" s="290" t="n"/>
+      <c r="L16" s="314" t="n"/>
       <c r="M16" s="185" t="n"/>
       <c r="N16" s="53" t="n"/>
     </row>
     <row r="17" ht="15" customFormat="1" customHeight="1" s="184">
       <c r="B17" s="211" t="n"/>
       <c r="C17" s="257" t="n"/>
-      <c r="D17" s="292" t="n"/>
+      <c r="D17" s="315" t="n"/>
       <c r="E17" s="179" t="n"/>
       <c r="F17" s="178" t="n"/>
       <c r="J17" s="211" t="n"/>
       <c r="K17" s="257" t="n"/>
-      <c r="L17" s="292" t="n"/>
+      <c r="L17" s="315" t="n"/>
       <c r="M17" s="179" t="n"/>
       <c r="N17" s="178" t="n"/>
     </row>
@@ -2945,26 +4727,26 @@
       <c r="F18" s="248" t="n"/>
       <c r="J18" s="211" t="n"/>
       <c r="K18" s="257" t="n"/>
-      <c r="L18" s="292" t="n"/>
+      <c r="L18" s="315" t="n"/>
       <c r="M18" s="179" t="n"/>
       <c r="N18" s="178" t="n"/>
     </row>
     <row r="19" ht="15" customFormat="1" customHeight="1" s="184">
       <c r="B19" s="81" t="n"/>
       <c r="C19" s="56" t="n"/>
-      <c r="D19" s="290" t="n"/>
+      <c r="D19" s="314" t="n"/>
       <c r="E19" s="185" t="n"/>
       <c r="F19" s="53" t="n"/>
       <c r="J19" s="274" t="n"/>
-      <c r="K19" s="275" t="n"/>
-      <c r="L19" s="275" t="n"/>
-      <c r="M19" s="275" t="n"/>
-      <c r="N19" s="276" t="n"/>
+      <c r="K19" s="284" t="n"/>
+      <c r="L19" s="284" t="n"/>
+      <c r="M19" s="284" t="n"/>
+      <c r="N19" s="275" t="n"/>
     </row>
     <row r="20" ht="15" customFormat="1" customHeight="1" s="184">
       <c r="B20" s="81" t="n"/>
       <c r="C20" s="56" t="n"/>
-      <c r="D20" s="290" t="n"/>
+      <c r="D20" s="314" t="n"/>
       <c r="E20" s="185" t="n"/>
       <c r="F20" s="53" t="n"/>
       <c r="J20" s="274" t="n"/>
@@ -2976,7 +4758,7 @@
     <row r="21" ht="15" customFormat="1" customHeight="1" s="184">
       <c r="B21" s="81" t="n"/>
       <c r="C21" s="56" t="n"/>
-      <c r="D21" s="290" t="n"/>
+      <c r="D21" s="314" t="n"/>
       <c r="E21" s="185" t="n"/>
       <c r="F21" s="53" t="n"/>
       <c r="J21" s="139" t="n"/>
@@ -2988,7 +4770,7 @@
     <row r="22" ht="15" customHeight="1" s="235">
       <c r="B22" s="81" t="n"/>
       <c r="C22" s="56" t="n"/>
-      <c r="D22" s="293" t="n"/>
+      <c r="D22" s="295" t="n"/>
       <c r="E22" s="186" t="n"/>
       <c r="F22" s="53" t="n"/>
       <c r="J22" s="139" t="n"/>
@@ -3000,7 +4782,7 @@
     <row r="23" ht="15" customFormat="1" customHeight="1" s="184">
       <c r="B23" s="211" t="n"/>
       <c r="C23" s="257" t="n"/>
-      <c r="D23" s="292" t="n"/>
+      <c r="D23" s="315" t="n"/>
       <c r="E23" s="179" t="n"/>
       <c r="F23" s="178" t="n"/>
       <c r="J23" s="139" t="n"/>

</xml_diff>